<commit_message>
Public release audit fixes
</commit_message>
<xml_diff>
--- a/data/source_data/SourceData_Figure4.xlsx
+++ b/data/source_data/SourceData_Figure4.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MATLABコード\小論文用\Figure\SourceData_Workbooks\書き換えた論文の番号対応ソース\投稿用\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12565B8A-434F-4DE2-81E4-C1D81585A04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294957B1-CA7D-40AF-9966-3E5B03BF0548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21255" yWindow="-8220" windowWidth="17280" windowHeight="8820" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22140" yWindow="-8610" windowWidth="21600" windowHeight="11235" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C_thetaopt" sheetId="3" r:id="rId1"/>

</xml_diff>